<commit_message>
HRMS employee onboarding utility
</commit_message>
<xml_diff>
--- a/Documents/MASTER_DATA/MasterData.xlsx
+++ b/Documents/MASTER_DATA/MasterData.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="9600" windowHeight="6800" firstSheet="12" activeTab="12"/>
+    <workbookView windowWidth="22188" windowHeight="9000" firstSheet="12" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="AppraisalStatusMaster" sheetId="1" r:id="rId1"/>
@@ -230,7 +230,7 @@
     <t>Birthday</t>
   </si>
   <si>
-    <t>New Joiner</t>
+    <t>New Joinee</t>
   </si>
   <si>
     <t>Work Anniversary</t>
@@ -941,7 +941,7 @@
     <cellStyle name="Percent" xfId="3" builtinId="5"/>
     <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
     <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
     <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
@@ -1467,7 +1467,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
@@ -1567,10 +1567,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="2" max="2" width="22.4454545454545" customWidth="1"/>
-    <col min="3" max="3" width="12.8909090909091" customWidth="1"/>
+    <col min="2" max="2" width="22.4444444444444" customWidth="1"/>
+    <col min="3" max="3" width="12.8888888888889" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1679,10 +1679,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14.5" outlineLevelRow="4" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="4" outlineLevelCol="1"/>
   <cols>
-    <col min="2" max="2" width="22.4454545454545" customWidth="1"/>
-    <col min="3" max="3" width="12.8909090909091" customWidth="1"/>
+    <col min="2" max="2" width="22.4444444444444" customWidth="1"/>
+    <col min="3" max="3" width="12.8888888888889" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1735,10 +1735,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="2" max="2" width="22.4454545454545" customWidth="1"/>
-    <col min="3" max="3" width="12.8909090909091" customWidth="1"/>
+    <col min="2" max="2" width="22.4444444444444" customWidth="1"/>
+    <col min="3" max="3" width="12.8888888888889" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1823,10 +1823,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14.5" outlineLevelRow="6" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="6" outlineLevelCol="1"/>
   <cols>
-    <col min="2" max="2" width="22.4454545454545" customWidth="1"/>
-    <col min="3" max="3" width="12.8909090909091" customWidth="1"/>
+    <col min="2" max="2" width="22.4444444444444" customWidth="1"/>
+    <col min="3" max="3" width="12.8888888888889" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -1875,10 +1875,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14.5" outlineLevelRow="4" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="4" outlineLevelCol="1"/>
   <cols>
-    <col min="1" max="1" width="6.21818181818182" customWidth="1"/>
-    <col min="2" max="2" width="17.1090909090909" customWidth="1"/>
+    <col min="1" max="1" width="6.22222222222222" customWidth="1"/>
+    <col min="2" max="2" width="17.1111111111111" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:2">
@@ -1931,9 +1931,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="2" max="2" width="17.4454545454545" customWidth="1"/>
+    <col min="2" max="2" width="17.4444444444444" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:2">
@@ -2050,9 +2050,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="2" max="2" width="20.6636363636364" customWidth="1"/>
+    <col min="2" max="2" width="20.6666666666667" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -2137,9 +2137,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="2" max="2" width="22.6636363636364" customWidth="1"/>
+    <col min="2" max="2" width="22.6666666666667" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -2224,9 +2224,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="1"/>
   <cols>
-    <col min="2" max="2" width="22.6636363636364" customWidth="1"/>
+    <col min="2" max="2" width="22.6666666666667" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -2271,9 +2271,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14.5" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="1"/>
   <cols>
-    <col min="2" max="2" width="33.2181818181818" customWidth="1"/>
+    <col min="2" max="2" width="33.2222222222222" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -2358,9 +2358,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14.5" outlineLevelRow="4" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="4" outlineLevelCol="1"/>
   <cols>
-    <col min="2" max="2" width="33.2181818181818" customWidth="1"/>
+    <col min="2" max="2" width="33.2222222222222" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -2413,7 +2413,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="1"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="1"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">

</xml_diff>